<commit_message>
[ADD] unificar ruta carpetas
</commit_message>
<xml_diff>
--- a/Plantilla_EMBARGO.xlsx
+++ b/Plantilla_EMBARGO.xlsx
@@ -1,16 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="5"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\Documents\Trabajo\JT\back-jt\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51F976EC-1DF6-44A2-9A22-230B67403702}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="EMBARGO" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="EMBARGO" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -22,290 +27,287 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="92">
   <si>
-    <t xml:space="preserve">NO ID DEMANDADO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TIPO DE PROCESO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOMBRE OFICIO INICIAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOMBRE OFICIO FINAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VALOR EMBARGO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NO. DE RADICADO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CUENTA BANCO AGRARIO / BANCO DEPÓSITO JUDICIAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOMBRE BANCO DEPÓSITO JUDICIAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOMBRE DEL SECRETARIO O FUNCIONARIO ENTE EMBARGANTE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CODIGO DE ALCANCE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CODIGO DE APLICACIÓN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TIPO LIMITE DE INEMBARGABILIDAD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TIPO DE APLICACIÓN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TIPO RESPUESTA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TIPO ID DEMANDADO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOMBRE DEMANDADO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TIPO ID DEMANDANTE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NO ID DEMANDANTE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOMBRE DEMANDANTE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOMBRE DEL ENTE EMBARGANTE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CIUDAD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CORREOS ELECTRÓNICOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LINK DE COLOCACIÓN DE RESPUESTA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PRODUCTOS A EMBARGAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SI ES CTA ESPECÍFICA, NO. DE CTA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PORCENTAJE A EMBARGAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PRODUCTOS A FUTURO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TIPO DOCUMENTO RECIBIDO EN EMAIL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TIPO DE REQUERIMIENTO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TIPO DE REQUERIMIENTO INEMBARGABLE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OBSERVACIONES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1023456789</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JUDICIAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1980-NOTIFICACION EMBARGO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20250232006224 DEL 241125 00000000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">68001400300520240075800</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BANCO AGRARIO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JUAN PEREZ GARCIA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1-INCO ID DDO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Art. 837-1ET - Aplican 25 SMLV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CONGELAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMAIL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PEDRO GOMEZ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">900123456</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIAN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JUZGADO 5 CIVIL MUNICIPAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BOGOTA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">notificaciones@juzgado.gov.co</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://ejemplo.gov.co/respuesta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TODOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INDIVIDUAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REQUERIMIENTO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REITERACION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9876543210</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COACTIVO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2100-EMBARGO CUENTAS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20250232006225 DEL 241125 00000000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11001400300520240012345</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MARIA LOPEZ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEBITAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FISICO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CARLOS RUIZ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">51234567</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ANA MARTINEZ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOBERNACION CUNDINAMARCA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MEDELLIN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AHORROS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">123456789</t>
-  </si>
-  <si>
-    <t xml:space="preserve">50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5551234567</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3050-RETENCION FONDOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20250232006226 DEL 241125 00000000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">76001400300520240098765</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BANCO AGRARIO S.A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ROBERTO DIAZ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LINK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LUIS FERNANDEZ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">800999888</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMPRESA XYZ SAS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JUZGADO 2 CIVIL CIRCUITO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CALI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://rama.gov.co/upload</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CORRIENTES</t>
+    <t>NO ID DEMANDADO</t>
+  </si>
+  <si>
+    <t>TIPO DE PROCESO</t>
+  </si>
+  <si>
+    <t>NOMBRE OFICIO INICIAL</t>
+  </si>
+  <si>
+    <t>NOMBRE OFICIO FINAL</t>
+  </si>
+  <si>
+    <t>VALOR EMBARGO</t>
+  </si>
+  <si>
+    <t>NO. DE RADICADO</t>
+  </si>
+  <si>
+    <t>CUENTA BANCO AGRARIO / BANCO DEPÓSITO JUDICIAL</t>
+  </si>
+  <si>
+    <t>NOMBRE BANCO DEPÓSITO JUDICIAL</t>
+  </si>
+  <si>
+    <t>NOMBRE DEL SECRETARIO O FUNCIONARIO ENTE EMBARGANTE</t>
+  </si>
+  <si>
+    <t>CODIGO DE ALCANCE</t>
+  </si>
+  <si>
+    <t>CODIGO DE APLICACIÓN</t>
+  </si>
+  <si>
+    <t>TIPO LIMITE DE INEMBARGABILIDAD</t>
+  </si>
+  <si>
+    <t>TIPO DE APLICACIÓN</t>
+  </si>
+  <si>
+    <t>TIPO RESPUESTA</t>
+  </si>
+  <si>
+    <t>TIPO ID DEMANDADO</t>
+  </si>
+  <si>
+    <t>NOMBRE DEMANDADO</t>
+  </si>
+  <si>
+    <t>TIPO ID DEMANDANTE</t>
+  </si>
+  <si>
+    <t>NO ID DEMANDANTE</t>
+  </si>
+  <si>
+    <t>NOMBRE DEMANDANTE</t>
+  </si>
+  <si>
+    <t>NOMBRE DEL ENTE EMBARGANTE</t>
+  </si>
+  <si>
+    <t>CIUDAD</t>
+  </si>
+  <si>
+    <t>CORREOS ELECTRÓNICOS</t>
+  </si>
+  <si>
+    <t>LINK DE COLOCACIÓN DE RESPUESTA</t>
+  </si>
+  <si>
+    <t>PRODUCTOS A EMBARGAR</t>
+  </si>
+  <si>
+    <t>SI ES CTA ESPECÍFICA, NO. DE CTA</t>
+  </si>
+  <si>
+    <t>PORCENTAJE A EMBARGAR</t>
+  </si>
+  <si>
+    <t>PRODUCTOS A FUTURO</t>
+  </si>
+  <si>
+    <t>TIPO DOCUMENTO RECIBIDO EN EMAIL</t>
+  </si>
+  <si>
+    <t>TIPO DE REQUERIMIENTO</t>
+  </si>
+  <si>
+    <t>TIPO DE REQUERIMIENTO INEMBARGABLE</t>
+  </si>
+  <si>
+    <t>OBSERVACIONES</t>
+  </si>
+  <si>
+    <t>1023456789</t>
+  </si>
+  <si>
+    <t>JUDICIAL</t>
+  </si>
+  <si>
+    <t>1980-NOTIFICACION EMBARGO</t>
+  </si>
+  <si>
+    <t>20250232006224 DEL 241125 00000000</t>
+  </si>
+  <si>
+    <t>68001400300520240075800</t>
+  </si>
+  <si>
+    <t>BANCO AGRARIO</t>
+  </si>
+  <si>
+    <t>JUAN PEREZ GARCIA</t>
+  </si>
+  <si>
+    <t>1-INCO ID DDO</t>
+  </si>
+  <si>
+    <t>01</t>
+  </si>
+  <si>
+    <t>Art. 837-1ET - Aplican 25 SMLV</t>
+  </si>
+  <si>
+    <t>CONGELAR</t>
+  </si>
+  <si>
+    <t>EMAIL</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>PEDRO GOMEZ</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>900123456</t>
+  </si>
+  <si>
+    <t>DIAN</t>
+  </si>
+  <si>
+    <t>JUZGADO 5 CIVIL MUNICIPAL</t>
+  </si>
+  <si>
+    <t>BOGOTA</t>
+  </si>
+  <si>
+    <t>notificaciones@juzgado.gov.co</t>
+  </si>
+  <si>
+    <t>https://ejemplo.gov.co/respuesta</t>
+  </si>
+  <si>
+    <t>TODOS</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t>SI</t>
+  </si>
+  <si>
+    <t>INDIVIDUAL</t>
+  </si>
+  <si>
+    <t>REQUERIMIENTO</t>
+  </si>
+  <si>
+    <t>REITERACION</t>
+  </si>
+  <si>
+    <t>9876543210</t>
+  </si>
+  <si>
+    <t>COACTIVO</t>
+  </si>
+  <si>
+    <t>2100-EMBARGO CUENTAS</t>
+  </si>
+  <si>
+    <t>20250232006225 DEL 241125 00000000</t>
+  </si>
+  <si>
+    <t>11001400300520240012345</t>
+  </si>
+  <si>
+    <t>MARIA LOPEZ</t>
+  </si>
+  <si>
+    <t>02</t>
+  </si>
+  <si>
+    <t>DEBITAR</t>
+  </si>
+  <si>
+    <t>FISICO</t>
+  </si>
+  <si>
+    <t>CARLOS RUIZ</t>
+  </si>
+  <si>
+    <t>51234567</t>
+  </si>
+  <si>
+    <t>ANA MARTINEZ</t>
+  </si>
+  <si>
+    <t>GOBERNACION CUNDINAMARCA</t>
+  </si>
+  <si>
+    <t>MEDELLIN</t>
+  </si>
+  <si>
+    <t>AHORROS</t>
+  </si>
+  <si>
+    <t>123456789</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>5551234567</t>
+  </si>
+  <si>
+    <t>3050-RETENCION FONDOS</t>
+  </si>
+  <si>
+    <t>20250232006226 DEL 241125 00000000</t>
+  </si>
+  <si>
+    <t>76001400300520240098765</t>
+  </si>
+  <si>
+    <t>BANCO AGRARIO S.A</t>
+  </si>
+  <si>
+    <t>ROBERTO DIAZ</t>
+  </si>
+  <si>
+    <t>03</t>
+  </si>
+  <si>
+    <t>LINK</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>LUIS FERNANDEZ</t>
+  </si>
+  <si>
+    <t>800999888</t>
+  </si>
+  <si>
+    <t>EMPRESA XYZ SAS</t>
+  </si>
+  <si>
+    <t>JUZGADO 2 CIVIL CIRCUITO</t>
+  </si>
+  <si>
+    <t>CALI</t>
+  </si>
+  <si>
+    <t>https://rama.gov.co/upload</t>
+  </si>
+  <si>
+    <t>CORRIENTES</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -314,26 +316,10 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -352,68 +338,44 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -472,13 +434,29 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF2F5496"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -520,12 +498,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -554,7 +532,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -572,7 +550,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -623,7 +601,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -641,55 +619,54 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AE4"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="31.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="0" width="25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="0" width="18"/>
+    <col min="1" max="2" width="19" customWidth="1"/>
+    <col min="3" max="3" width="31.77734375" customWidth="1"/>
+    <col min="4" max="4" width="23" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
+    <col min="7" max="7" width="50" customWidth="1"/>
+    <col min="8" max="8" width="34" customWidth="1"/>
+    <col min="9" max="9" width="55" customWidth="1"/>
+    <col min="10" max="10" width="21" customWidth="1"/>
+    <col min="11" max="11" width="24" customWidth="1"/>
+    <col min="12" max="12" width="35" customWidth="1"/>
+    <col min="13" max="13" width="22" customWidth="1"/>
+    <col min="14" max="14" width="18" customWidth="1"/>
+    <col min="15" max="15" width="21" customWidth="1"/>
+    <col min="16" max="16" width="20" customWidth="1"/>
+    <col min="17" max="17" width="22" customWidth="1"/>
+    <col min="18" max="18" width="20" customWidth="1"/>
+    <col min="19" max="19" width="21" customWidth="1"/>
+    <col min="20" max="20" width="30" customWidth="1"/>
+    <col min="21" max="21" width="18" customWidth="1"/>
+    <col min="22" max="22" width="24" customWidth="1"/>
+    <col min="23" max="23" width="35" customWidth="1"/>
+    <col min="24" max="24" width="24" customWidth="1"/>
+    <col min="25" max="25" width="36" customWidth="1"/>
+    <col min="26" max="26" width="25" customWidth="1"/>
+    <col min="27" max="27" width="22" customWidth="1"/>
+    <col min="28" max="28" width="36" customWidth="1"/>
+    <col min="29" max="29" width="25" customWidth="1"/>
+    <col min="30" max="30" width="38" customWidth="1"/>
+    <col min="31" max="31" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:31" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -784,7 +761,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>31</v>
       </c>
@@ -797,13 +774,13 @@
       <c r="D2" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="2">
         <v>5000000</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="G2" s="2">
         <v>110014189005</v>
       </c>
       <c r="H2" s="2" t="s">
@@ -870,14 +847,14 @@
       <c r="AC2" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="AD2" s="2" t="n">
+      <c r="AD2" s="2">
         <v>0</v>
       </c>
       <c r="AE2" s="2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>58</v>
       </c>
@@ -890,13 +867,13 @@
       <c r="D3" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="2">
         <v>3000000</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="G3" s="2">
         <v>110014189006</v>
       </c>
       <c r="H3" s="2" t="s">
@@ -965,14 +942,14 @@
       <c r="AC3" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="AD3" s="2" t="n">
+      <c r="AD3" s="2">
         <v>0</v>
       </c>
       <c r="AE3" s="2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>76</v>
       </c>
@@ -985,13 +962,13 @@
       <c r="D4" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="2">
         <v>10000000</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="G4" s="2">
         <v>110014189007</v>
       </c>
       <c r="H4" s="2" t="s">
@@ -1060,7 +1037,7 @@
       <c r="AC4" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="AD4" s="2" t="n">
+      <c r="AD4" s="2">
         <v>0</v>
       </c>
       <c r="AE4" s="2" t="s">
@@ -1068,12 +1045,7 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>